<commit_message>
Release v2.2.0: Email Intelligence — CHANGELOG + DevEconomics
Add the 2.2.0 "Built with no code" changelog block and update the
DevEconomics workbook + narrative for the Email Intelligence feature
(38 activities; ~$21 est, reconcile via /cost). Fold the prior
Gmail/Drive release into the foundation baseline so the App Total stays
correct (~5.2 KLOC, ~$72 est to date).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deveconomics/DigitalSecretary-DevEconomics.xlsx
+++ b/docs/deveconomics/DigitalSecretary-DevEconomics.xlsx
@@ -874,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -953,12 +953,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>Requirements</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Read CLAUDE.md; locate solution &amp; memory</t>
+          <t>Brainstorm uses; draft email-intelligence requirements (Groups A-K)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Read/Glob</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -977,13 +977,13 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -992,7 +992,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>orient</t>
+          <t>BA/product doc</t>
         </is>
       </c>
     </row>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>Requirements</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Study EmailDownloader (control, IMAP, settings, helpers)</t>
+          <t>Add timeline / documents / progress / HTML-report requirements</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1026,10 +1026,10 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12000</v>
+        <v>4000</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>3</v>
@@ -1039,11 +1039,7 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>model to clone</t>
-        </is>
-      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1056,7 +1052,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Read contract, ADDING_A_FEATURE, Directory.Build.props</t>
+          <t>Read CLAUDE.md, contract, EmailDownloader, build.ps1, docgen, tests (~20 reads)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1075,20 +1071,24 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>6000</v>
+        <v>40000</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>one-time pattern learning</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Read unit + QA tests and QA harness</t>
+          <t>Read ADDING_A_FEATURE, check_docs, build_excel_docs, coverage.runsettings</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1120,20 +1120,24 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>7000</v>
+        <v>18000</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>quality gates</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1141,48 +1145,42 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Read build.ps1, docgen scripts, check_docs</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>A - LLM tokens</t>
+          <t>Verify dotnet/python/nuget/git + MimeKit cache</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>B - Local ($0)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Bash</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>14000</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
       <c r="H6" s="4" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>quality gates</t>
-        </is>
-      </c>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1190,12 +1188,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Read requirements/user-guide/journal/manual template/DocShots</t>
+          <t>Author models + MailText + EmailParser + ArchiveScanner</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1205,7 +1203,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1214,13 +1212,13 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>13000</v>
+        <v>9000</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.13</v>
+        <v>0.35</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -1229,7 +1227,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>docs pipeline</t>
+          <t>MimeKit + .txt</t>
         </is>
       </c>
     </row>
@@ -1239,46 +1237,44 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Decide</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Ask 3 scoping questions (IMAP vs API, OAuth, export fmt)</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>A - LLM tokens</t>
+          <t>Compile parsing slice</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>B - Local ($0)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>AskUserQuestion</t>
+          <t>dotnet build</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>2000</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
       <c r="H8" s="4" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>blocking decisions</t>
+          <t>8.7s</t>
         </is>
       </c>
     </row>
@@ -1288,39 +1284,41 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Verify toolchain (dotnet/python/nuget/git/openpyxl)</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Author 9 analyzer classes (dedupe/contacts/identity/signature/metrics/graph/topics/timeline/classify)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>PowerShell</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>12000</v>
+      </c>
       <c r="H9" s="4" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1331,12 +1329,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Build Gmail</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Author 9 Gmail files (module, control, IMAP, naming, scanner, settings, manifest, FEATURE)</t>
+          <t>Fix nullable + CA1859 warnings</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1346,7 +1344,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1355,24 +1353,20 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>14000</v>
+        <v>1500</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.45</v>
+        <v>0.04</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>521 LOC</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1380,42 +1374,48 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Build Gmail</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Add project to solution + unit-test reference</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Author exporters + HTML report generator + pipeline + settings + UI + module</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>dotnet sln/add</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>16000</v>
+      </c>
       <c r="H11" s="4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.2</v>
+        <v>9</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>report has embedded CSS/JS</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Build Gmail</t>
+          <t>Build P1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Compile Gmail feature (0 warnings)</t>
+          <t>Compile full feature (0 warnings)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1451,18 +1451,14 @@
         <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>measured</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>8.4s</t>
-        </is>
-      </c>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1470,12 +1466,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Tests P1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Author pure logic (export formats, file naming, settings)</t>
+          <t>Author 14 unit-test files + fixtures</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1494,24 +1490,20 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.18</v>
+        <v>0.35</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>testable, no Google dep</t>
-        </is>
-      </c>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1519,41 +1511,39 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Tests P1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Author csproj / manifest / module</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>A - LLM tokens</t>
+          <t>Add feature reference to unit-test project</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>B - Local ($0)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>dotnet add reference</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>2000</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
       <c r="H14" s="4" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
@@ -1564,22 +1554,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Tests P1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Add Google.Apis.Drive.v3 + restore</t>
+          <t>Run unit tests (121)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>B+C - Local+net ($0)</t>
+          <t>B - Local ($0)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>dotnet add package</t>
+          <t>dotnet test</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1592,7 +1582,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
@@ -1601,7 +1591,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>NuGet download 5.9s</t>
+          <t>7s</t>
         </is>
       </c>
     </row>
@@ -1611,12 +1601,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Author OAuth + Drive API downloader + control + FEATURE</t>
+          <t>Author FEATURE.md + user-guide doc</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1635,24 +1625,20 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.4</v>
+        <v>0.14</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>512 LOC</t>
-        </is>
-      </c>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1660,12 +1646,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Docgen</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Simplify download helper</t>
+          <t>Edit build_excel_docs (37 reqs + 16 trace) + check_docs EI id regex</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1684,13 +1670,13 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1500</v>
+        <v>8000</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.04</v>
+        <v>0.22</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -1705,12 +1691,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Docgen</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Add to solution + unit-test reference</t>
+          <t>Regenerate xlsx + run check_docs + secret scan</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1720,7 +1706,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>dotnet sln/add</t>
+          <t>python</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1733,7 +1719,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1748,12 +1734,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Gate</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Compile Drive (2 analyzer warnings)</t>
+          <t>Full quality gate</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1763,7 +1749,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>dotnet build</t>
+          <t>build.ps1 -All</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1776,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -1785,7 +1771,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>6.3s</t>
+          <t>PASS, 92%</t>
         </is>
       </c>
     </row>
@@ -1795,12 +1781,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Gate</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Fix CA1859 + CA2016 warnings</t>
+          <t>Append DEVELOPMENT_JOURNAL phase</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1819,13 +1805,13 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1840,44 +1826,46 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Build Drive</t>
+          <t>Append</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Recompile Drive (0 warnings)</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Add AnalysisMode + ScanAndParse/AnalyzeCore refactor (EI-I4)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>dotnet build</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>7000</v>
+      </c>
       <c r="H21" s="4" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.04</v>
+        <v>5</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>2.5s</t>
+          <t>consolidate archives</t>
         </is>
       </c>
     </row>
@@ -1887,12 +1875,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Append</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Author 4 unit-test files (Gmail + Drive logic)</t>
+          <t>Wire Append checkbox into the UI</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1902,7 +1890,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1911,24 +1899,20 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>6000</v>
+        <v>2000</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>233 LOC</t>
-        </is>
-      </c>
+      <c r="K22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1936,12 +1920,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Append</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Add settings round-trips + QA private-dependency tests</t>
+          <t>Author MessageStore + append/overwrite tests</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1951,7 +1935,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1960,13 +1944,13 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -1981,12 +1965,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Append</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Build full solution</t>
+          <t>Run tests (125)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1996,7 +1980,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>dotnet build</t>
+          <t>dotnet test</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2009,18 +1993,14 @@
         <v>0</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.21</v>
+        <v>0.1</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>measured</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>12.5s, 0 warn</t>
-        </is>
-      </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2028,12 +2008,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Append</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Run unit tests</t>
+          <t>Register EI-I4 + regenerate + gate</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2043,7 +2023,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>dotnet test</t>
+          <t>python/build.ps1</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2056,7 +2036,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.75</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
@@ -2065,7 +2045,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>85 pass, 4s</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2075,44 +2055,46 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Build P3</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Run QA automation</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Author SentimentLexicon + ToneAnalyzer + LifeDataExtractor + DocumentLibrary + model fields</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>dotnet test</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>9000</v>
+      </c>
       <c r="H26" s="4" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.02</v>
+        <v>6</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>17 pass, 1s</t>
+          <t>E2, F1-F4, F7</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2104,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Build P3</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Author requirement + user-guide docs (4)</t>
+          <t>Wire pipeline + CSV exporters + JSON + 2 HTML tabs</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2137,7 +2119,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2152,7 +2134,7 @@
         <v>0.2</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
@@ -2167,12 +2149,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Build P3</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Update REQUIREMENTS / USER_GUIDE indexes</t>
+          <t>Author 3 analyzer test files</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2182,7 +2164,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2191,13 +2173,13 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0.05</v>
+        <v>0.14</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2212,41 +2194,39 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Docgen</t>
+          <t>Build P3</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Edit build_excel_docs.py + check_docs.py (GML/GDR rows + ID regex)</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>A - LLM tokens</t>
+          <t>Run tests (147)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>B - Local ($0)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>dotnet test</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>5000</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
       <c r="H29" s="4" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>2.5</v>
+        <v>0.1</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
@@ -2257,12 +2237,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Docgen</t>
+          <t>Build P3</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Regenerate requirements + traceability xlsx</t>
+          <t>Register E2/F + regenerate + gate</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2272,7 +2252,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>python/build.ps1</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2285,7 +2265,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
@@ -2294,7 +2274,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>56 req, 37 trace</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -2304,44 +2284,46 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Docgen</t>
+          <t>Build P4</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Run docs consistency checker</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Author XlsxWriter (dependency-free OOXML) + WorkbookExporter + wire pipeline</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>python check_docs</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>6000</v>
+      </c>
       <c r="H31" s="4" t="n">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0.05</v>
+        <v>4</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>caught 24 expected</t>
+          <t>native .xlsx</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2333,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Build P4</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Edit manual template (TOC + 2 sections) + DocShots seed</t>
+          <t>Hoist header arrays (CA1861)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2375,13 +2357,13 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>0.12</v>
+        <v>0.03</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
@@ -2396,46 +2378,44 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Build P4</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Generate screenshots</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>Author XlsxWriter tests</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>dotnet run DocShots</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>2500</v>
+      </c>
       <c r="H33" s="4" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>8 PNGs</t>
-        </is>
-      </c>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2443,12 +2423,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Build P4</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Build single-file HTML manual</t>
+          <t>Validate .xlsx with openpyxl (throwaway runner)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2458,7 +2438,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>build-user-manual.ps1</t>
+          <t>dotnet run + python</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2471,7 +2451,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03</v>
+        <v>0.4</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -2480,7 +2460,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>192KB, clean</t>
+          <t>3 sheets, typed numbers</t>
         </is>
       </c>
     </row>
@@ -2490,12 +2470,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Build P4</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Re-run consistency checker</t>
+          <t>Register EI-H7 + regenerate + gate</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2505,7 +2485,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>python check_docs</t>
+          <t>python/build.ps1</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2518,7 +2498,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
@@ -2527,7 +2507,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>0 errors</t>
+          <t>PASS, 91.9%</t>
         </is>
       </c>
     </row>
@@ -2537,12 +2517,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Commit</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Append DEVELOPMENT_JOURNAL phase</t>
+          <t>Fix test fixtures to example.com (secret gate) + stage</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2552,7 +2532,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Bash/Edit</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2561,10 +2541,10 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="I36" s="5" t="n">
         <v>1</v>
@@ -2574,7 +2554,11 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>74 leaks -&gt; 0</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2582,12 +2566,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Commit</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Full quality gate</t>
+          <t>Commit feature + xlsx (pre-commit gate x2)</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2597,7 +2581,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>build.ps1 -All</t>
+          <t>git commit</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2610,7 +2594,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
@@ -2619,7 +2603,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>PASS, 72.9% cov</t>
+          <t>84d97dd, 3562b3d</t>
         </is>
       </c>
     </row>
@@ -2629,48 +2613,42 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Fix coverage.runsettings exclusions</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>A - LLM tokens</t>
+          <t>Push main to origin</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>B+C - Local+net ($0)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>git push</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="n">
-        <v>1500</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n"/>
       <c r="H38" s="4" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>exclude network classes</t>
-        </is>
-      </c>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2678,166 +2656,74 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Re-run gate with -MinCoverage 80</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
+          <t>DevEconomics + CHANGELOG + cut release</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>A - LLM tokens</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>build.ps1 -All</t>
+          <t>Write/Edit</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>6000</v>
+      </c>
       <c r="H39" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>0.7</v>
+        <v>5</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>PASS, 89.9%</t>
+          <t>this release entry</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Cleanliness scan (mojibake) + git status</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Grep/git</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>measured</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>0 mojibake</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Commit</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Commit + pre-commit gate</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>B - Local ($0)</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>git commit</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>measured</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>1df66a4</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>TOTAL (direct, sum of activities)</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="7">
-        <f>SUM(G2:G41)</f>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="7">
+        <f>SUM(G2:G39)</f>
         <v/>
       </c>
-      <c r="H42" s="8">
-        <f>SUM(H2:H41)</f>
+      <c r="H40" s="8">
+        <f>SUM(H2:H39)</f>
         <v/>
       </c>
-      <c r="I42" s="9">
-        <f>SUM(I2:I41)</f>
+      <c r="I40" s="9">
+        <f>SUM(I2:I39)</f>
         <v/>
       </c>
-      <c r="J42" s="2" t="n"/>
-      <c r="K42" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
@@ -2970,12 +2856,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Foundation (host + first 4 features + quality/docs/CI/release infra)</t>
+          <t>Prior releases (host + 6 features + quality/docs/CI/release infra, through v2.1.0)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19..20</t>
+          <t>2026-06-19..22</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2987,15 +2873,15 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n">
-        <v>1.7</v>
+        <v>2.73</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>2000000</v>
+        <v>2121000</v>
       </c>
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n">
-        <v>45</v>
+        <v>50.5</v>
       </c>
       <c r="L2" s="4" t="n"/>
       <c r="M2" s="4">
@@ -3004,22 +2890,22 @@
       </c>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n">
-        <v>720</v>
+        <v>768</v>
       </c>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="4" t="n">
-        <v>26.47</v>
+        <v>18.5</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>ROUGH estimate - phases 1-17 predate DevEconomics tracking (not logged live).</t>
+          <t>ROUGH estimate: phases 1-17 predate DevEconomics tracking; includes the tracked Gmail/Drive release (v2.1.0, ~$5.50).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Gmail + Google Drive downloaders</t>
+          <t>Email Intelligence</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -3033,28 +2919,28 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1.03</v>
+        <v>2.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>121000</v>
+        <v>182700</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2.73</v>
+        <v>5.1</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>2.77</v>
+        <v>16</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>5.5</v>
+        <v>21.1</v>
       </c>
       <c r="L3" s="4" t="n"/>
       <c r="M3" s="4">
@@ -3062,18 +2948,18 @@
         <v/>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3.51</v>
+        <v>5.12</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>48.01</v>
+        <v>99.72</v>
       </c>
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="4" t="n">
-        <v>5.34</v>
+        <v>8.44</v>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Estimate; reconcile ACTUAL via /cost. Excludes the DevEconomics report + cost analysis.</t>
+          <t>Estimate; reconcile ACTUAL via /cost. Spans 3 increments (foundation+report, append, tone/life-data/docs, xlsx).</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3132,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Token/cost for LLM rows are ESTIMATES (the model can't read its own meter). Local times are MEASURED from command output where captured. Per-feature ACTUAL cost comes from /cost (Claude Code) or the Anthropic Console - fill columns J/N in Feature Summary, then re-run.</t>
+          <t>Token/cost for LLM rows are ESTIMATES (the model can't read its own meter). Local times are MEASURED from command output where captured. Per-feature ACTUAL cost comes from /cost (Claude Code) or the Anthropic Console - fill columns L/P in Feature Summary, then re-run.</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3144,7 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>40 activities (21 LLM / 19 local|remote); ~$5.5 est; ~48.01 min est (~3.51 min measured local compute).</t>
+          <t>38 activities (23 LLM / 15 local|remote); ~$21.1 est; ~99.72 min est (~5.12 min measured local compute).</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3156,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>~2.73 prod KLOC; ~$50.5 est; ~12.8 h est. Foundation portion is a ROUGH pre-tracking estimate.</t>
+          <t>~5.23 prod KLOC; ~$71.6 est; ~14.5 h est. Foundation portion is a ROUGH pre-tracking estimate.</t>
         </is>
       </c>
     </row>

</xml_diff>